<commit_message>
Restore original layout and fix component refactoring
- Fixed mini calendars: restored original compact format in left sidebar
- Fixed navbar: restored search and filters to navbar (not sidebar)
- Maintained clean build with no lint warnings
- BigCal.tsx still over 2000 lines but functionality preserved
- Created component extraction foundation (GridView, FilterPanel, MiniCalendarPanel)
- Updated CSV test data to 2025 dates for current testing
- All major features working: color system, status handling, import/export
</commit_message>
<xml_diff>
--- a/test-data/BigCal-Speed-Test-20-Events.xlsx
+++ b/test-data/BigCal-Speed-Test-20-Events.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\BigCal\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{040B83FB-0BE6-4AA7-8326-18F9FBCFE54C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E61CE60-621C-41B4-88D7-B3119A32B5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60930" yWindow="405" windowWidth="21600" windowHeight="11295" xr2:uid="{86CCFAF1-B6FD-4512-B421-0217CBDDF04B}"/>
+    <workbookView xWindow="34020" yWindow="1425" windowWidth="21600" windowHeight="11295" xr2:uid="{86CCFAF1-B6FD-4512-B421-0217CBDDF04B}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="53">
   <si>
     <t>Title</t>
   </si>
@@ -1086,9 +1086,6 @@
       <c r="E2" t="s">
         <v>8</v>
       </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -1146,9 +1143,6 @@
       <c r="E5" t="s">
         <v>19</v>
       </c>
-      <c r="F5" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -1186,9 +1180,6 @@
       <c r="E7" t="s">
         <v>8</v>
       </c>
-      <c r="F7" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -1246,9 +1237,6 @@
       <c r="E10" t="s">
         <v>19</v>
       </c>
-      <c r="F10" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -1266,9 +1254,6 @@
       <c r="E11" t="s">
         <v>22</v>
       </c>
-      <c r="F11" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -1286,9 +1271,6 @@
       <c r="E12" t="s">
         <v>8</v>
       </c>
-      <c r="F12" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -1306,9 +1288,6 @@
       <c r="E13" t="s">
         <v>12</v>
       </c>
-      <c r="F13" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -1326,9 +1305,6 @@
       <c r="E14" t="s">
         <v>16</v>
       </c>
-      <c r="F14" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -1346,9 +1322,6 @@
       <c r="E15" t="s">
         <v>19</v>
       </c>
-      <c r="F15" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -1366,11 +1339,8 @@
       <c r="E16" t="s">
         <v>22</v>
       </c>
-      <c r="F16" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -1386,11 +1356,8 @@
       <c r="E17" t="s">
         <v>8</v>
       </c>
-      <c r="F17" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>45</v>
       </c>
@@ -1406,11 +1373,8 @@
       <c r="E18" t="s">
         <v>12</v>
       </c>
-      <c r="F18" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>47</v>
       </c>
@@ -1426,11 +1390,8 @@
       <c r="E19" t="s">
         <v>16</v>
       </c>
-      <c r="F19" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>49</v>
       </c>
@@ -1446,11 +1407,8 @@
       <c r="E20" t="s">
         <v>19</v>
       </c>
-      <c r="F20" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>51</v>
       </c>
@@ -1465,9 +1423,6 @@
       </c>
       <c r="E21" t="s">
         <v>22</v>
-      </c>
-      <c r="F21" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>